<commit_message>
Menu: swap Dahi Vada and Shahi Tukda between Thu and Fri week-1 dinners
</commit_message>
<xml_diff>
--- a/sources/August-Sept Menu Updated.xlsx
+++ b/sources/August-Sept Menu Updated.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dell\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kuriangeorge/Library/Containers/net.whatsapp.WhatsApp/Data/tmp/documents/96E43F60-98DC-4FF1-8E7E-ECF90BEFF262/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{340A53BE-7C69-4150-84E8-EA4F7FBE1731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90A53A6A-3A77-A74B-B501-A100FB1FBA6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1" sheetId="1" r:id="rId1"/>
@@ -179,9 +179,6 @@
     <t>Egg Masala, Kadhai Paneer, Dal Tadka, Steam rice, chapati, Salad, Pickle, Besan Barfi</t>
   </si>
   <si>
-    <t xml:space="preserve"> Rajasthani Dahi, Sev Tamatar, Steam Rice, Chapati, Salad, Pickle, Dahi Vada</t>
-  </si>
-  <si>
     <t>Baigan Masala, Mix Veg, Dal Kolhapuri, Steam Rice, Papad, Chapati, Rasam, Masala Chhach</t>
   </si>
   <si>
@@ -224,13 +221,16 @@
     <t>Misal Pav,Aloo Sabudana khichdi , Farsan, Bread, Jam, Butter, Tea Coffee</t>
   </si>
   <si>
-    <t>Tomato Rice, Matki Gravy,Veg Kolhapuri, Chapati, Salad, Onion Raita, Shahi Tukda</t>
-  </si>
-  <si>
     <t>Dal makhani, Jeera Rice, Methi Aloo Sabzi, Chapati, Salad, Pickle, Jalebi</t>
   </si>
   <si>
     <t>Tomato Bharta, tawa vegetable, Dal Tadka, Steam rice, Chapati, Salad, Pickle, Dry Fruit Sheera</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rajasthani Dahi, Sev Tamatar, Steam Rice, Chapati, Salad, Pickle, Shahi Tukda</t>
+  </si>
+  <si>
+    <t>Tomato Rice, Matki Gravy,Veg Kolhapuri, Chapati, Salad, Onion Raita, Dahi Vada</t>
   </si>
 </sst>
 </file>
@@ -699,17 +699,17 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="54" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="54" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="20.77734375" style="6" customWidth="1"/>
-    <col min="2" max="2" width="51.88671875" style="7" customWidth="1"/>
+    <col min="1" max="1" width="20.796875" style="6" customWidth="1"/>
+    <col min="2" max="2" width="51.796875" style="7" customWidth="1"/>
     <col min="3" max="3" width="77" style="7" customWidth="1"/>
-    <col min="4" max="4" width="50.88671875" style="7" customWidth="1"/>
-    <col min="5" max="5" width="70.109375" style="7" customWidth="1"/>
+    <col min="4" max="4" width="50.796875" style="7" customWidth="1"/>
+    <col min="5" max="5" width="70.19921875" style="7" customWidth="1"/>
     <col min="6" max="16384" width="9" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="5" customFormat="1" ht="29.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="5" customFormat="1" ht="29.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="8" t="s">
         <v>26</v>
       </c>
@@ -718,7 +718,7 @@
       <c r="D1" s="8"/>
       <c r="E1" s="8"/>
     </row>
-    <row r="2" spans="1:5" s="6" customFormat="1" ht="26.55" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" s="6" customFormat="1" ht="26.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -735,7 +735,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
@@ -746,30 +746,30 @@
         <v>21</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
@@ -780,13 +780,13 @@
         <v>42</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
@@ -800,10 +800,10 @@
         <v>33</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
@@ -817,10 +817,10 @@
         <v>45</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
@@ -828,7 +828,7 @@
         <v>35</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>46</v>
@@ -837,7 +837,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
@@ -851,10 +851,10 @@
         <v>13</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" s="5" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" s="5" customFormat="1" ht="27.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="8" t="s">
         <v>27</v>
       </c>
@@ -863,7 +863,7 @@
       <c r="D10" s="8"/>
       <c r="E10" s="8"/>
     </row>
-    <row r="11" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="3" t="s">
         <v>5</v>
       </c>
@@ -877,10 +877,10 @@
         <v>22</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="40" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>14</v>
       </c>
@@ -888,16 +888,16 @@
         <v>23</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>7</v>
       </c>
@@ -914,7 +914,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>8</v>
       </c>
@@ -922,7 +922,7 @@
         <v>40</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>48</v>
@@ -931,15 +931,15 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>28</v>
@@ -948,7 +948,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>10</v>
       </c>
@@ -956,7 +956,7 @@
         <v>23</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>49</v>
@@ -965,7 +965,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>11</v>
       </c>
@@ -988,14 +988,14 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.22" right="0.2" top="0.36" bottom="0.48" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="8" scale="84" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="8" scale="85" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F2C8D21-48BE-4A46-B08C-8B938A4A8070}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>